<commit_message>
validação e ajustes para bom funcionamento do relatório, adição do agrupamento de lista técnicas, agora a lista técnica não é mais atualizada uma vez por mês e sim todo dia.
</commit_message>
<xml_diff>
--- a/temp/diversos/Aluminio.xlsx
+++ b/temp/diversos/Aluminio.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="66">
   <si>
     <t>ACIONADOR DA TRAVA ELETROMAGNÉTICA</t>
   </si>
@@ -40,18 +40,12 @@
     <t>ARANHA INFERIOR SUGGAR COM PÉS</t>
   </si>
   <si>
-    <t>ARANHA INFERIOR TANQUINHO MODELO NOVO M4</t>
-  </si>
-  <si>
     <t>ARANHA SUP. DO DESLIZANTE FURO M5</t>
   </si>
   <si>
     <t>ARANHA SUPERIOR SUGGAR</t>
   </si>
   <si>
-    <t>ARANHA SUPERIOR TANQUINHO MODELO NOVO M5</t>
-  </si>
-  <si>
     <t>BASE AGL FECH. ELETROÍMÃ AL150 / AL180 - BRUTO</t>
   </si>
   <si>
@@ -70,12 +64,6 @@
     <t>CAIXA DA TRAVA ELETROMAGNÉTICA - ALUMÍNIO</t>
   </si>
   <si>
-    <t>CANTONEIRA ATRAQUE ELETROIMA AL150 / AL180 - BRUTO</t>
-  </si>
-  <si>
-    <t>CANTONEIRA BASE ELETROIMA AL150 / AL180 - BRUTO</t>
-  </si>
-  <si>
     <t>CARCAÇA DA FECHADURA MINI SMART (ADAPTAÇÃO NOVO MINI MOTOR)</t>
   </si>
   <si>
@@ -109,15 +97,12 @@
     <t>FIM DE CURSO MECANICO DE ALUMÍNIO</t>
   </si>
   <si>
-    <t>FUNDO ALUMINIO FECHO PV200RF2I - BRUTO</t>
+    <t>FUNDO ALUMINIO LINGUETA PV200RF2I - BRUTO</t>
   </si>
   <si>
     <t>PC</t>
   </si>
   <si>
-    <t>FUNDO ALUMINIO LINGUETA PV200RF2I - BRUTO</t>
-  </si>
-  <si>
     <t>FUNDO DO PAINEL RX200/ RX500</t>
   </si>
   <si>
@@ -206,9 +191,6 @@
   </si>
   <si>
     <t>PINO DESTRAVAMENTO MOTOR DZ INDUSTRIAL</t>
-  </si>
-  <si>
-    <t>PROTEÇÃO CANTONEIRA DA BASE ELETROIMA AL150 / AL180 - BRUTO</t>
   </si>
   <si>
     <t>PS-ST SAE-060 AGL 16,8MM 2P (SOMENTE MOTOR P/ INDUSTRIALIZAÇÃO)</t>
@@ -328,7 +310,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col customWidth="1" width="7.33203125" min="1" max="1"/>
@@ -519,7 +501,7 @@
         <v>3</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>8580</v>
+        <v>7846</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>0</v>
@@ -536,7 +518,7 @@
     </row>
     <row r="7" customHeight="1" ht="15" spans="1:10">
       <c r="A7" s="1" t="n">
-        <v>813530</v>
+        <v>813238</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>9</v>
@@ -551,7 +533,7 @@
         <v>3</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>860</v>
+        <v>2950</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>0</v>
@@ -568,7 +550,7 @@
     </row>
     <row r="8" customHeight="1" ht="15" spans="1:10">
       <c r="A8" s="1" t="n">
-        <v>813238</v>
+        <v>813604</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>10</v>
@@ -583,7 +565,7 @@
         <v>3</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>2950</v>
+        <v>2991</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>0</v>
@@ -600,7 +582,7 @@
     </row>
     <row r="9" customHeight="1" ht="15" spans="1:10">
       <c r="A9" s="1" t="n">
-        <v>813604</v>
+        <v>701125</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>11</v>
@@ -615,7 +597,7 @@
         <v>3</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>4458</v>
+        <v>4015</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>0</v>
@@ -632,7 +614,7 @@
     </row>
     <row r="10" customHeight="1" ht="15" spans="1:10">
       <c r="A10" s="1" t="n">
-        <v>813531</v>
+        <v>813241</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>12</v>
@@ -647,7 +629,7 @@
         <v>3</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>860</v>
+        <v>72</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>0</v>
@@ -664,7 +646,7 @@
     </row>
     <row r="11" customHeight="1" ht="15" spans="1:10">
       <c r="A11" s="1" t="n">
-        <v>701125</v>
+        <v>813199</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>13</v>
@@ -679,7 +661,7 @@
         <v>3</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>4015</v>
+        <v>262</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>0</v>
@@ -696,7 +678,7 @@
     </row>
     <row r="12" customHeight="1" ht="15" spans="1:10">
       <c r="A12" s="1" t="n">
-        <v>813241</v>
+        <v>813153</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>14</v>
@@ -711,7 +693,7 @@
         <v>3</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>72</v>
+        <v>194</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>0</v>
@@ -728,7 +710,7 @@
     </row>
     <row r="13" customHeight="1" ht="15" spans="1:10">
       <c r="A13" s="1" t="n">
-        <v>813199</v>
+        <v>701107</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>15</v>
@@ -743,7 +725,7 @@
         <v>3</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>262</v>
+        <v>2705</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>0</v>
@@ -760,7 +742,7 @@
     </row>
     <row r="14" customHeight="1" ht="15" spans="1:10">
       <c r="A14" s="1" t="n">
-        <v>813153</v>
+        <v>807119</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>16</v>
@@ -775,7 +757,7 @@
         <v>3</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>194</v>
+        <v>520</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>0</v>
@@ -792,7 +774,7 @@
     </row>
     <row r="15" customHeight="1" ht="15" spans="1:10">
       <c r="A15" s="1" t="n">
-        <v>701107</v>
+        <v>807162</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>17</v>
@@ -807,7 +789,7 @@
         <v>3</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>2705</v>
+        <v>700</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>0</v>
@@ -824,7 +806,7 @@
     </row>
     <row r="16" customHeight="1" ht="15" spans="1:10">
       <c r="A16" s="1" t="n">
-        <v>807119</v>
+        <v>813271</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>18</v>
@@ -839,7 +821,7 @@
         <v>3</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>520</v>
+        <v>548</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>0</v>
@@ -856,7 +838,7 @@
     </row>
     <row r="17" customHeight="1" ht="15" spans="1:10">
       <c r="A17" s="1" t="n">
-        <v>701120</v>
+        <v>813258</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>19</v>
@@ -871,7 +853,7 @@
         <v>3</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>4033</v>
+        <v>1428</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>0</v>
@@ -888,7 +870,7 @@
     </row>
     <row r="18" customHeight="1" ht="15" spans="1:10">
       <c r="A18" s="1" t="n">
-        <v>701122</v>
+        <v>807158</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>20</v>
@@ -903,7 +885,7 @@
         <v>3</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>5174</v>
+        <v>3133</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>0</v>
@@ -920,7 +902,7 @@
     </row>
     <row r="19" customHeight="1" ht="15" spans="1:10">
       <c r="A19" s="1" t="n">
-        <v>807162</v>
+        <v>813265</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>21</v>
@@ -935,7 +917,7 @@
         <v>3</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>700</v>
+        <v>1161</v>
       </c>
       <c r="G19" s="3" t="n">
         <v>0</v>
@@ -952,7 +934,7 @@
     </row>
     <row r="20" customHeight="1" ht="15" spans="1:10">
       <c r="A20" s="1" t="n">
-        <v>813271</v>
+        <v>813311</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>22</v>
@@ -967,7 +949,7 @@
         <v>3</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>548</v>
+        <v>5524</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>0</v>
@@ -984,7 +966,7 @@
     </row>
     <row r="21" customHeight="1" ht="15" spans="1:10">
       <c r="A21" s="1" t="n">
-        <v>813258</v>
+        <v>813310</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>23</v>
@@ -999,7 +981,7 @@
         <v>3</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>1428</v>
+        <v>11745</v>
       </c>
       <c r="G21" s="3" t="n">
         <v>0</v>
@@ -1016,7 +998,7 @@
     </row>
     <row r="22" customHeight="1" ht="15" spans="1:10">
       <c r="A22" s="1" t="n">
-        <v>807158</v>
+        <v>813243</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>24</v>
@@ -1031,7 +1013,7 @@
         <v>3</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>3133</v>
+        <v>409</v>
       </c>
       <c r="G22" s="3" t="n">
         <v>0</v>
@@ -1048,7 +1030,7 @@
     </row>
     <row r="23" customHeight="1" ht="15" spans="1:10">
       <c r="A23" s="1" t="n">
-        <v>813265</v>
+        <v>813037</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>25</v>
@@ -1063,7 +1045,7 @@
         <v>3</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>1161</v>
+        <v>1457</v>
       </c>
       <c r="G23" s="3" t="n">
         <v>0</v>
@@ -1080,7 +1062,7 @@
     </row>
     <row r="24" customHeight="1" ht="15" spans="1:10">
       <c r="A24" s="1" t="n">
-        <v>813311</v>
+        <v>701189</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>26</v>
@@ -1095,7 +1077,7 @@
         <v>3</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>5524</v>
+        <v>1705</v>
       </c>
       <c r="G24" s="3" t="n">
         <v>0</v>
@@ -1112,7 +1094,7 @@
     </row>
     <row r="25" customHeight="1" ht="15" spans="1:10">
       <c r="A25" s="1" t="n">
-        <v>813310</v>
+        <v>813623</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>27</v>
@@ -1127,7 +1109,7 @@
         <v>3</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>11745</v>
+        <v>3952</v>
       </c>
       <c r="G25" s="3" t="n">
         <v>0</v>
@@ -1144,13 +1126,13 @@
     </row>
     <row r="26" customHeight="1" ht="15" spans="1:10">
       <c r="A26" s="1" t="n">
-        <v>813243</v>
+        <v>707029</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>2</v>
@@ -1159,7 +1141,7 @@
         <v>3</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>409</v>
+        <v>1072</v>
       </c>
       <c r="G26" s="3" t="n">
         <v>0</v>
@@ -1176,10 +1158,10 @@
     </row>
     <row r="27" customHeight="1" ht="15" spans="1:10">
       <c r="A27" s="1" t="n">
-        <v>813037</v>
+        <v>807155</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>1</v>
@@ -1191,7 +1173,7 @@
         <v>3</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>1457</v>
+        <v>540</v>
       </c>
       <c r="G27" s="3" t="n">
         <v>0</v>
@@ -1208,10 +1190,10 @@
     </row>
     <row r="28" customHeight="1" ht="15" spans="1:10">
       <c r="A28" s="1" t="n">
-        <v>701189</v>
+        <v>807203</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>1</v>
@@ -1223,7 +1205,7 @@
         <v>3</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>1705</v>
+        <v>1005</v>
       </c>
       <c r="G28" s="3" t="n">
         <v>0</v>
@@ -1240,10 +1222,10 @@
     </row>
     <row r="29" customHeight="1" ht="15" spans="1:10">
       <c r="A29" s="1" t="n">
-        <v>813623</v>
+        <v>813146</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>1</v>
@@ -1255,7 +1237,7 @@
         <v>3</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>3952</v>
+        <v>12167</v>
       </c>
       <c r="G29" s="3" t="n">
         <v>0</v>
@@ -1272,22 +1254,22 @@
     </row>
     <row r="30" customHeight="1" ht="15" spans="1:10">
       <c r="A30" s="1" t="n">
-        <v>707030</v>
+        <v>203004</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>1072</v>
+        <v>118.118</v>
       </c>
       <c r="G30" s="3" t="n">
         <v>0</v>
@@ -1304,22 +1286,22 @@
     </row>
     <row r="31" customHeight="1" ht="15" spans="1:10">
       <c r="A31" s="1" t="n">
-        <v>707029</v>
+        <v>203006</v>
       </c>
       <c r="B31" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C31" s="1" t="s">
-        <v>33</v>
-      </c>
       <c r="D31" s="2" t="s">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>1072</v>
+        <v>42464.762</v>
       </c>
       <c r="G31" s="3" t="n">
         <v>0</v>
@@ -1336,13 +1318,13 @@
     </row>
     <row r="32" customHeight="1" ht="15" spans="1:10">
       <c r="A32" s="1" t="n">
-        <v>807155</v>
+        <v>707023</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>2</v>
@@ -1351,7 +1333,7 @@
         <v>3</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>540</v>
+        <v>1654</v>
       </c>
       <c r="G32" s="3" t="n">
         <v>0</v>
@@ -1368,10 +1350,10 @@
     </row>
     <row r="33" customHeight="1" ht="15" spans="1:10">
       <c r="A33" s="1" t="n">
-        <v>807203</v>
+        <v>707022</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>1</v>
@@ -1383,7 +1365,7 @@
         <v>3</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>1005</v>
+        <v>3050</v>
       </c>
       <c r="G33" s="3" t="n">
         <v>0</v>
@@ -1400,10 +1382,10 @@
     </row>
     <row r="34" customHeight="1" ht="15" spans="1:10">
       <c r="A34" s="1" t="n">
-        <v>813146</v>
+        <v>813513</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>1</v>
@@ -1415,7 +1397,7 @@
         <v>3</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>8220</v>
+        <v>11</v>
       </c>
       <c r="G34" s="3" t="n">
         <v>0</v>
@@ -1432,22 +1414,22 @@
     </row>
     <row r="35" customHeight="1" ht="15" spans="1:10">
       <c r="A35" s="1" t="n">
-        <v>203004</v>
+        <v>813512</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>2924.786</v>
+        <v>80</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>0</v>
@@ -1464,22 +1446,22 @@
     </row>
     <row r="36" customHeight="1" ht="15" spans="1:10">
       <c r="A36" s="1" t="n">
-        <v>203006</v>
+        <v>412090</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>25697.078</v>
+        <v>3183</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>0</v>
@@ -1496,13 +1478,13 @@
     </row>
     <row r="37" customHeight="1" ht="15" spans="1:10">
       <c r="A37" s="1" t="n">
-        <v>707023</v>
+        <v>412168</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>2</v>
@@ -1511,7 +1493,7 @@
         <v>3</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>1654</v>
+        <v>150</v>
       </c>
       <c r="G37" s="3" t="n">
         <v>0</v>
@@ -1528,7 +1510,7 @@
     </row>
     <row r="38" customHeight="1" ht="15" spans="1:10">
       <c r="A38" s="1" t="n">
-        <v>707022</v>
+        <v>412388</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>44</v>
@@ -1543,7 +1525,7 @@
         <v>3</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>3050</v>
+        <v>13</v>
       </c>
       <c r="G38" s="3" t="n">
         <v>0</v>
@@ -1560,7 +1542,7 @@
     </row>
     <row r="39" customHeight="1" ht="15" spans="1:10">
       <c r="A39" s="1" t="n">
-        <v>813513</v>
+        <v>412380</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>45</v>
@@ -1575,7 +1557,7 @@
         <v>3</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>11</v>
+        <v>145</v>
       </c>
       <c r="G39" s="3" t="n">
         <v>0</v>
@@ -1592,7 +1574,7 @@
     </row>
     <row r="40" customHeight="1" ht="15" spans="1:10">
       <c r="A40" s="1" t="n">
-        <v>813512</v>
+        <v>412043</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>46</v>
@@ -1607,7 +1589,7 @@
         <v>3</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>80</v>
+        <v>2496</v>
       </c>
       <c r="G40" s="3" t="n">
         <v>0</v>
@@ -1624,7 +1606,7 @@
     </row>
     <row r="41" customHeight="1" ht="15" spans="1:10">
       <c r="A41" s="1" t="n">
-        <v>412090</v>
+        <v>813448</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>47</v>
@@ -1639,7 +1621,7 @@
         <v>3</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>3183</v>
+        <v>5300</v>
       </c>
       <c r="G41" s="3" t="n">
         <v>0</v>
@@ -1656,7 +1638,7 @@
     </row>
     <row r="42" customHeight="1" ht="15" spans="1:10">
       <c r="A42" s="1" t="n">
-        <v>412168</v>
+        <v>412094</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>48</v>
@@ -1671,7 +1653,7 @@
         <v>3</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>150</v>
+        <v>14466</v>
       </c>
       <c r="G42" s="3" t="n">
         <v>0</v>
@@ -1688,7 +1670,7 @@
     </row>
     <row r="43" customHeight="1" ht="15" spans="1:10">
       <c r="A43" s="1" t="n">
-        <v>412388</v>
+        <v>412107</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>49</v>
@@ -1703,7 +1685,7 @@
         <v>3</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>13</v>
+        <v>1629</v>
       </c>
       <c r="G43" s="3" t="n">
         <v>0</v>
@@ -1720,7 +1702,7 @@
     </row>
     <row r="44" customHeight="1" ht="15" spans="1:10">
       <c r="A44" s="1" t="n">
-        <v>412380</v>
+        <v>412051</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>50</v>
@@ -1735,7 +1717,7 @@
         <v>3</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>145</v>
+        <v>1915</v>
       </c>
       <c r="G44" s="3" t="n">
         <v>0</v>
@@ -1752,7 +1734,7 @@
     </row>
     <row r="45" customHeight="1" ht="15" spans="1:10">
       <c r="A45" s="1" t="n">
-        <v>412043</v>
+        <v>412387</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>51</v>
@@ -1767,7 +1749,7 @@
         <v>3</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>2496</v>
+        <v>191</v>
       </c>
       <c r="G45" s="3" t="n">
         <v>0</v>
@@ -1784,7 +1766,7 @@
     </row>
     <row r="46" customHeight="1" ht="15" spans="1:10">
       <c r="A46" s="1" t="n">
-        <v>813448</v>
+        <v>412109</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>52</v>
@@ -1799,7 +1781,7 @@
         <v>3</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>4682</v>
+        <v>819</v>
       </c>
       <c r="G46" s="3" t="n">
         <v>0</v>
@@ -1816,7 +1798,7 @@
     </row>
     <row r="47" customHeight="1" ht="15" spans="1:10">
       <c r="A47" s="1" t="n">
-        <v>412094</v>
+        <v>412092</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>53</v>
@@ -1831,7 +1813,7 @@
         <v>3</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>5734</v>
+        <v>2553</v>
       </c>
       <c r="G47" s="3" t="n">
         <v>0</v>
@@ -1848,7 +1830,7 @@
     </row>
     <row r="48" customHeight="1" ht="15" spans="1:10">
       <c r="A48" s="1" t="n">
-        <v>412107</v>
+        <v>412366</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>54</v>
@@ -1863,7 +1845,7 @@
         <v>3</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>1629</v>
+        <v>1283</v>
       </c>
       <c r="G48" s="3" t="n">
         <v>0</v>
@@ -1880,7 +1862,7 @@
     </row>
     <row r="49" customHeight="1" ht="15" spans="1:10">
       <c r="A49" s="1" t="n">
-        <v>412051</v>
+        <v>412075</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>55</v>
@@ -1895,7 +1877,7 @@
         <v>3</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>1915</v>
+        <v>910</v>
       </c>
       <c r="G49" s="3" t="n">
         <v>0</v>
@@ -1912,7 +1894,7 @@
     </row>
     <row r="50" customHeight="1" ht="15" spans="1:10">
       <c r="A50" s="1" t="n">
-        <v>412387</v>
+        <v>412111</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>56</v>
@@ -1927,7 +1909,7 @@
         <v>3</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>191</v>
+        <v>345</v>
       </c>
       <c r="G50" s="3" t="n">
         <v>0</v>
@@ -1944,7 +1926,7 @@
     </row>
     <row r="51" customHeight="1" ht="15" spans="1:10">
       <c r="A51" s="1" t="n">
-        <v>412109</v>
+        <v>412089</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>57</v>
@@ -1959,7 +1941,7 @@
         <v>3</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>819</v>
+        <v>1100</v>
       </c>
       <c r="G51" s="3" t="n">
         <v>0</v>
@@ -1976,7 +1958,7 @@
     </row>
     <row r="52" customHeight="1" ht="15" spans="1:10">
       <c r="A52" s="1" t="n">
-        <v>412092</v>
+        <v>412126</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>58</v>
@@ -1991,7 +1973,7 @@
         <v>3</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>548</v>
+        <v>21</v>
       </c>
       <c r="G52" s="3" t="n">
         <v>0</v>
@@ -2008,7 +1990,7 @@
     </row>
     <row r="53" customHeight="1" ht="15" spans="1:10">
       <c r="A53" s="1" t="n">
-        <v>412366</v>
+        <v>701159</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>59</v>
@@ -2023,7 +2005,7 @@
         <v>3</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>1283</v>
+        <v>438</v>
       </c>
       <c r="G53" s="3" t="n">
         <v>0</v>
@@ -2040,7 +2022,7 @@
     </row>
     <row r="54" customHeight="1" ht="15" spans="1:10">
       <c r="A54" s="1" t="n">
-        <v>412075</v>
+        <v>412139</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>60</v>
@@ -2055,7 +2037,7 @@
         <v>3</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>910</v>
+        <v>520</v>
       </c>
       <c r="G54" s="3" t="n">
         <v>0</v>
@@ -2072,7 +2054,7 @@
     </row>
     <row r="55" customHeight="1" ht="15" spans="1:10">
       <c r="A55" s="1" t="n">
-        <v>412111</v>
+        <v>412108</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>61</v>
@@ -2087,7 +2069,7 @@
         <v>3</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>345</v>
+        <v>600</v>
       </c>
       <c r="G55" s="3" t="n">
         <v>0</v>
@@ -2104,7 +2086,7 @@
     </row>
     <row r="56" customHeight="1" ht="15" spans="1:10">
       <c r="A56" s="1" t="n">
-        <v>412089</v>
+        <v>412110</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>62</v>
@@ -2119,7 +2101,7 @@
         <v>3</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>1100</v>
+        <v>600</v>
       </c>
       <c r="G56" s="3" t="n">
         <v>0</v>
@@ -2136,7 +2118,7 @@
     </row>
     <row r="57" customHeight="1" ht="15" spans="1:10">
       <c r="A57" s="1" t="n">
-        <v>412126</v>
+        <v>412033</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>63</v>
@@ -2151,7 +2133,7 @@
         <v>3</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>21</v>
+        <v>600</v>
       </c>
       <c r="G57" s="3" t="n">
         <v>0</v>
@@ -2168,7 +2150,7 @@
     </row>
     <row r="58" customHeight="1" ht="15" spans="1:10">
       <c r="A58" s="1" t="n">
-        <v>701159</v>
+        <v>412037</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>64</v>
@@ -2183,7 +2165,7 @@
         <v>3</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>438</v>
+        <v>600</v>
       </c>
       <c r="G58" s="3" t="n">
         <v>0</v>
@@ -2200,7 +2182,7 @@
     </row>
     <row r="59" customHeight="1" ht="15" spans="1:10">
       <c r="A59" s="1" t="n">
-        <v>701123</v>
+        <v>813467</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>65</v>
@@ -2215,7 +2197,7 @@
         <v>3</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>1981</v>
+        <v>1271</v>
       </c>
       <c r="G59" s="3" t="n">
         <v>0</v>
@@ -2227,198 +2209,6 @@
         <v>0</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" customHeight="1" ht="15" spans="1:10">
-      <c r="A60" s="1" t="n">
-        <v>412139</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F60" s="3" t="n">
-        <v>520</v>
-      </c>
-      <c r="G60" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H60" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I60" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J60" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" customHeight="1" ht="15" spans="1:10">
-      <c r="A61" s="1" t="n">
-        <v>412108</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F61" s="3" t="n">
-        <v>600</v>
-      </c>
-      <c r="G61" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H61" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I61" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J61" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" customHeight="1" ht="15" spans="1:10">
-      <c r="A62" s="1" t="n">
-        <v>412110</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F62" s="3" t="n">
-        <v>600</v>
-      </c>
-      <c r="G62" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H62" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I62" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J62" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" customHeight="1" ht="15" spans="1:10">
-      <c r="A63" s="1" t="n">
-        <v>412033</v>
-      </c>
-      <c r="B63" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F63" s="3" t="n">
-        <v>600</v>
-      </c>
-      <c r="G63" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H63" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I63" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J63" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" customHeight="1" ht="15" spans="1:10">
-      <c r="A64" s="1" t="n">
-        <v>412037</v>
-      </c>
-      <c r="B64" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E64" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F64" s="3" t="n">
-        <v>600</v>
-      </c>
-      <c r="G64" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H64" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I64" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J64" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" customHeight="1" ht="15" spans="1:10">
-      <c r="A65" s="1" t="n">
-        <v>813467</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E65" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F65" s="3" t="n">
-        <v>1271</v>
-      </c>
-      <c r="G65" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H65" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I65" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J65" s="3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
criação do arquivo check_relatório que faz a checagem de atualização do relatório, assim já extraindo os dados automáticamente
</commit_message>
<xml_diff>
--- a/temp/diversos/Aluminio.xlsx
+++ b/temp/diversos/Aluminio.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="71">
   <si>
     <t>ACIONADOR DA TRAVA ELETROMAGNÉTICA</t>
   </si>
@@ -40,12 +40,18 @@
     <t>ARANHA INFERIOR SUGGAR COM PÉS</t>
   </si>
   <si>
+    <t>ARANHA INFERIOR TANQUINHO MODELO NOVO M4</t>
+  </si>
+  <si>
     <t>ARANHA SUP. DO DESLIZANTE FURO M5</t>
   </si>
   <si>
     <t>ARANHA SUPERIOR SUGGAR</t>
   </si>
   <si>
+    <t>ARANHA SUPERIOR TANQUINHO MODELO NOVO M5</t>
+  </si>
+  <si>
     <t>BASE AGL FECH. ELETROÍMÃ AL150 / AL180 - BRUTO</t>
   </si>
   <si>
@@ -89,6 +95,13 @@
   </si>
   <si>
     <t>ENGRENAGEM EXTERNA MOTOR 17 DENTES</t>
+  </si>
+  <si>
+    <t>ENGRENAGEM EXTERNA 17D PARA EIXO ESTAMPADO TRINO LIGHT/300
+</t>
+  </si>
+  <si>
+    <t>AGL ELETRONICOS</t>
   </si>
   <si>
     <t>ESPELHO DO BATENTE DA FECHADURA RX100 / RX200 / RX500 - BRUTO</t>
@@ -313,7 +326,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col customWidth="1" width="7.33203125" min="1" max="1"/>
@@ -440,7 +453,7 @@
         <v>3</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>4792</v>
+        <v>9792</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>0</v>
@@ -504,7 +517,7 @@
         <v>3</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>7846</v>
+        <v>5952</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>0</v>
@@ -521,7 +534,7 @@
     </row>
     <row r="7" customHeight="1" ht="15" spans="1:10">
       <c r="A7" s="1" t="n">
-        <v>813238</v>
+        <v>813530</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>9</v>
@@ -536,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>2950</v>
+        <v>5000</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>0</v>
@@ -553,7 +566,7 @@
     </row>
     <row r="8" customHeight="1" ht="15" spans="1:10">
       <c r="A8" s="1" t="n">
-        <v>813604</v>
+        <v>813238</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>10</v>
@@ -568,7 +581,7 @@
         <v>3</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>2188</v>
+        <v>7950</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>0</v>
@@ -585,7 +598,7 @@
     </row>
     <row r="9" customHeight="1" ht="15" spans="1:10">
       <c r="A9" s="1" t="n">
-        <v>701125</v>
+        <v>813604</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>11</v>
@@ -600,7 +613,7 @@
         <v>3</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>4015</v>
+        <v>650</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>0</v>
@@ -617,7 +630,7 @@
     </row>
     <row r="10" customHeight="1" ht="15" spans="1:10">
       <c r="A10" s="1" t="n">
-        <v>813241</v>
+        <v>813531</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>12</v>
@@ -632,7 +645,7 @@
         <v>3</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>72</v>
+        <v>5000</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>0</v>
@@ -649,7 +662,7 @@
     </row>
     <row r="11" customHeight="1" ht="15" spans="1:10">
       <c r="A11" s="1" t="n">
-        <v>813199</v>
+        <v>701125</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>13</v>
@@ -664,7 +677,7 @@
         <v>3</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>262</v>
+        <v>4015</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>0</v>
@@ -681,7 +694,7 @@
     </row>
     <row r="12" customHeight="1" ht="15" spans="1:10">
       <c r="A12" s="1" t="n">
-        <v>813153</v>
+        <v>813241</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>14</v>
@@ -696,7 +709,7 @@
         <v>3</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>194</v>
+        <v>72</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>0</v>
@@ -713,7 +726,7 @@
     </row>
     <row r="13" customHeight="1" ht="15" spans="1:10">
       <c r="A13" s="1" t="n">
-        <v>701107</v>
+        <v>813199</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>15</v>
@@ -728,7 +741,7 @@
         <v>3</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>2705</v>
+        <v>262</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>0</v>
@@ -745,7 +758,7 @@
     </row>
     <row r="14" customHeight="1" ht="15" spans="1:10">
       <c r="A14" s="1" t="n">
-        <v>807119</v>
+        <v>813153</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>16</v>
@@ -760,7 +773,7 @@
         <v>3</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>520</v>
+        <v>194</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>0</v>
@@ -777,7 +790,7 @@
     </row>
     <row r="15" customHeight="1" ht="15" spans="1:10">
       <c r="A15" s="1" t="n">
-        <v>807162</v>
+        <v>701107</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>17</v>
@@ -792,7 +805,7 @@
         <v>3</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>700</v>
+        <v>2705</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>0</v>
@@ -809,7 +822,7 @@
     </row>
     <row r="16" customHeight="1" ht="15" spans="1:10">
       <c r="A16" s="1" t="n">
-        <v>813271</v>
+        <v>807119</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>18</v>
@@ -824,7 +837,7 @@
         <v>3</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>548</v>
+        <v>520</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>0</v>
@@ -841,7 +854,7 @@
     </row>
     <row r="17" customHeight="1" ht="15" spans="1:10">
       <c r="A17" s="1" t="n">
-        <v>813258</v>
+        <v>807162</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>19</v>
@@ -856,7 +869,7 @@
         <v>3</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>1428</v>
+        <v>700</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>0</v>
@@ -873,7 +886,7 @@
     </row>
     <row r="18" customHeight="1" ht="15" spans="1:10">
       <c r="A18" s="1" t="n">
-        <v>807158</v>
+        <v>813271</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>20</v>
@@ -888,7 +901,7 @@
         <v>3</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>3133</v>
+        <v>15</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>0</v>
@@ -905,7 +918,7 @@
     </row>
     <row r="19" customHeight="1" ht="15" spans="1:10">
       <c r="A19" s="1" t="n">
-        <v>813265</v>
+        <v>813258</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>21</v>
@@ -920,7 +933,7 @@
         <v>3</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>1161</v>
+        <v>1428</v>
       </c>
       <c r="G19" s="3" t="n">
         <v>0</v>
@@ -937,7 +950,7 @@
     </row>
     <row r="20" customHeight="1" ht="15" spans="1:10">
       <c r="A20" s="1" t="n">
-        <v>813311</v>
+        <v>807158</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>22</v>
@@ -952,7 +965,7 @@
         <v>3</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>5524</v>
+        <v>3133</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>0</v>
@@ -969,7 +982,7 @@
     </row>
     <row r="21" customHeight="1" ht="15" spans="1:10">
       <c r="A21" s="1" t="n">
-        <v>813310</v>
+        <v>813265</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>23</v>
@@ -984,7 +997,7 @@
         <v>3</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>11745</v>
+        <v>1161</v>
       </c>
       <c r="G21" s="3" t="n">
         <v>0</v>
@@ -1001,7 +1014,7 @@
     </row>
     <row r="22" customHeight="1" ht="15" spans="1:10">
       <c r="A22" s="1" t="n">
-        <v>813243</v>
+        <v>813311</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>24</v>
@@ -1016,7 +1029,7 @@
         <v>3</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>409</v>
+        <v>5524</v>
       </c>
       <c r="G22" s="3" t="n">
         <v>0</v>
@@ -1033,7 +1046,7 @@
     </row>
     <row r="23" customHeight="1" ht="15" spans="1:10">
       <c r="A23" s="1" t="n">
-        <v>813037</v>
+        <v>813310</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>25</v>
@@ -1048,7 +1061,7 @@
         <v>3</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>1457</v>
+        <v>11745</v>
       </c>
       <c r="G23" s="3" t="n">
         <v>0</v>
@@ -1065,7 +1078,7 @@
     </row>
     <row r="24" customHeight="1" ht="15" spans="1:10">
       <c r="A24" s="1" t="n">
-        <v>701189</v>
+        <v>813243</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>26</v>
@@ -1080,7 +1093,7 @@
         <v>3</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>1705</v>
+        <v>409</v>
       </c>
       <c r="G24" s="3" t="n">
         <v>0</v>
@@ -1097,7 +1110,7 @@
     </row>
     <row r="25" customHeight="1" ht="15" spans="1:10">
       <c r="A25" s="1" t="n">
-        <v>813623</v>
+        <v>813037</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>27</v>
@@ -1112,7 +1125,7 @@
         <v>3</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>3952</v>
+        <v>1457</v>
       </c>
       <c r="G25" s="3" t="n">
         <v>0</v>
@@ -1129,22 +1142,22 @@
     </row>
     <row r="26" customHeight="1" ht="15" spans="1:10">
       <c r="A26" s="1" t="n">
-        <v>707029</v>
+        <v>813096</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C26" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>3</v>
-      </c>
       <c r="F26" s="3" t="n">
-        <v>1072</v>
+        <v>9688</v>
       </c>
       <c r="G26" s="3" t="n">
         <v>0</v>
@@ -1161,7 +1174,7 @@
     </row>
     <row r="27" customHeight="1" ht="15" spans="1:10">
       <c r="A27" s="1" t="n">
-        <v>807155</v>
+        <v>701189</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>30</v>
@@ -1176,7 +1189,7 @@
         <v>3</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>540</v>
+        <v>1705</v>
       </c>
       <c r="G27" s="3" t="n">
         <v>0</v>
@@ -1193,7 +1206,7 @@
     </row>
     <row r="28" customHeight="1" ht="15" spans="1:10">
       <c r="A28" s="1" t="n">
-        <v>807203</v>
+        <v>813623</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>31</v>
@@ -1208,7 +1221,7 @@
         <v>3</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>1005</v>
+        <v>3952</v>
       </c>
       <c r="G28" s="3" t="n">
         <v>0</v>
@@ -1225,13 +1238,13 @@
     </row>
     <row r="29" customHeight="1" ht="15" spans="1:10">
       <c r="A29" s="1" t="n">
-        <v>813146</v>
+        <v>707029</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>32</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>2</v>
@@ -1240,7 +1253,7 @@
         <v>3</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>12167</v>
+        <v>1072</v>
       </c>
       <c r="G29" s="3" t="n">
         <v>0</v>
@@ -1257,22 +1270,22 @@
     </row>
     <row r="30" customHeight="1" ht="15" spans="1:10">
       <c r="A30" s="1" t="n">
-        <v>203004</v>
+        <v>807155</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>118.118</v>
+        <v>540</v>
       </c>
       <c r="G30" s="3" t="n">
         <v>0</v>
@@ -1289,22 +1302,22 @@
     </row>
     <row r="31" customHeight="1" ht="15" spans="1:10">
       <c r="A31" s="1" t="n">
-        <v>203006</v>
+        <v>807203</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>42464.762</v>
+        <v>1005</v>
       </c>
       <c r="G31" s="3" t="n">
         <v>0</v>
@@ -1321,13 +1334,13 @@
     </row>
     <row r="32" customHeight="1" ht="15" spans="1:10">
       <c r="A32" s="1" t="n">
-        <v>707023</v>
+        <v>813146</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>2</v>
@@ -1336,7 +1349,7 @@
         <v>3</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>1654</v>
+        <v>12167</v>
       </c>
       <c r="G32" s="3" t="n">
         <v>0</v>
@@ -1353,22 +1366,22 @@
     </row>
     <row r="33" customHeight="1" ht="15" spans="1:10">
       <c r="A33" s="1" t="n">
-        <v>707022</v>
+        <v>203004</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C33" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>2</v>
-      </c>
       <c r="E33" s="1" t="s">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>3050</v>
+        <v>118.117959</v>
       </c>
       <c r="G33" s="3" t="n">
         <v>0</v>
@@ -1385,22 +1398,22 @@
     </row>
     <row r="34" customHeight="1" ht="15" spans="1:10">
       <c r="A34" s="1" t="n">
-        <v>813513</v>
+        <v>203006</v>
       </c>
       <c r="B34" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E34" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C34" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>3</v>
-      </c>
       <c r="F34" s="3" t="n">
-        <v>11</v>
+        <v>46037.262</v>
       </c>
       <c r="G34" s="3" t="n">
         <v>0</v>
@@ -1417,13 +1430,13 @@
     </row>
     <row r="35" customHeight="1" ht="15" spans="1:10">
       <c r="A35" s="1" t="n">
-        <v>813512</v>
+        <v>707023</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>2</v>
@@ -1432,7 +1445,7 @@
         <v>3</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>80</v>
+        <v>1654</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>0</v>
@@ -1449,10 +1462,10 @@
     </row>
     <row r="36" customHeight="1" ht="15" spans="1:10">
       <c r="A36" s="1" t="n">
-        <v>412090</v>
+        <v>707022</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>1</v>
@@ -1464,7 +1477,7 @@
         <v>3</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>3183</v>
+        <v>3050</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>0</v>
@@ -1481,10 +1494,10 @@
     </row>
     <row r="37" customHeight="1" ht="15" spans="1:10">
       <c r="A37" s="1" t="n">
-        <v>412168</v>
+        <v>813513</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>1</v>
@@ -1496,7 +1509,7 @@
         <v>3</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>150</v>
+        <v>11</v>
       </c>
       <c r="G37" s="3" t="n">
         <v>0</v>
@@ -1513,10 +1526,10 @@
     </row>
     <row r="38" customHeight="1" ht="15" spans="1:10">
       <c r="A38" s="1" t="n">
-        <v>412388</v>
+        <v>813512</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>1</v>
@@ -1528,7 +1541,7 @@
         <v>3</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>13</v>
+        <v>80</v>
       </c>
       <c r="G38" s="3" t="n">
         <v>0</v>
@@ -1545,10 +1558,10 @@
     </row>
     <row r="39" customHeight="1" ht="15" spans="1:10">
       <c r="A39" s="1" t="n">
-        <v>412380</v>
+        <v>412090</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>1</v>
@@ -1560,7 +1573,7 @@
         <v>3</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>145</v>
+        <v>3183</v>
       </c>
       <c r="G39" s="3" t="n">
         <v>0</v>
@@ -1577,10 +1590,10 @@
     </row>
     <row r="40" customHeight="1" ht="15" spans="1:10">
       <c r="A40" s="1" t="n">
-        <v>412043</v>
+        <v>412168</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>1</v>
@@ -1592,7 +1605,7 @@
         <v>3</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>2496</v>
+        <v>150</v>
       </c>
       <c r="G40" s="3" t="n">
         <v>0</v>
@@ -1609,10 +1622,10 @@
     </row>
     <row r="41" customHeight="1" ht="15" spans="1:10">
       <c r="A41" s="1" t="n">
-        <v>813448</v>
+        <v>412388</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>1</v>
@@ -1624,7 +1637,7 @@
         <v>3</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>5300</v>
+        <v>13</v>
       </c>
       <c r="G41" s="3" t="n">
         <v>0</v>
@@ -1641,10 +1654,10 @@
     </row>
     <row r="42" customHeight="1" ht="15" spans="1:10">
       <c r="A42" s="1" t="n">
-        <v>412094</v>
+        <v>412380</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>1</v>
@@ -1656,7 +1669,7 @@
         <v>3</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>12396</v>
+        <v>145</v>
       </c>
       <c r="G42" s="3" t="n">
         <v>0</v>
@@ -1673,10 +1686,10 @@
     </row>
     <row r="43" customHeight="1" ht="15" spans="1:10">
       <c r="A43" s="1" t="n">
-        <v>412107</v>
+        <v>412043</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>1</v>
@@ -1688,7 +1701,7 @@
         <v>3</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>1629</v>
+        <v>2496</v>
       </c>
       <c r="G43" s="3" t="n">
         <v>0</v>
@@ -1705,10 +1718,10 @@
     </row>
     <row r="44" customHeight="1" ht="15" spans="1:10">
       <c r="A44" s="1" t="n">
-        <v>813443</v>
+        <v>813448</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>1</v>
@@ -1720,7 +1733,7 @@
         <v>3</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>624</v>
+        <v>5300</v>
       </c>
       <c r="G44" s="3" t="n">
         <v>0</v>
@@ -1737,10 +1750,10 @@
     </row>
     <row r="45" customHeight="1" ht="15" spans="1:10">
       <c r="A45" s="1" t="n">
-        <v>412051</v>
+        <v>412094</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>1</v>
@@ -1752,7 +1765,7 @@
         <v>3</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>1915</v>
+        <v>11031</v>
       </c>
       <c r="G45" s="3" t="n">
         <v>0</v>
@@ -1769,10 +1782,10 @@
     </row>
     <row r="46" customHeight="1" ht="15" spans="1:10">
       <c r="A46" s="1" t="n">
-        <v>412387</v>
+        <v>412107</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>1</v>
@@ -1784,7 +1797,7 @@
         <v>3</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>191</v>
+        <v>1629</v>
       </c>
       <c r="G46" s="3" t="n">
         <v>0</v>
@@ -1801,10 +1814,10 @@
     </row>
     <row r="47" customHeight="1" ht="15" spans="1:10">
       <c r="A47" s="1" t="n">
-        <v>412109</v>
+        <v>813443</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>1</v>
@@ -1816,7 +1829,7 @@
         <v>3</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>819</v>
+        <v>3024</v>
       </c>
       <c r="G47" s="3" t="n">
         <v>0</v>
@@ -1833,10 +1846,10 @@
     </row>
     <row r="48" customHeight="1" ht="15" spans="1:10">
       <c r="A48" s="1" t="n">
-        <v>412092</v>
+        <v>412051</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>1</v>
@@ -1848,7 +1861,7 @@
         <v>3</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>2553</v>
+        <v>1915</v>
       </c>
       <c r="G48" s="3" t="n">
         <v>0</v>
@@ -1865,10 +1878,10 @@
     </row>
     <row r="49" customHeight="1" ht="15" spans="1:10">
       <c r="A49" s="1" t="n">
-        <v>412366</v>
+        <v>412387</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>1</v>
@@ -1880,7 +1893,7 @@
         <v>3</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>1283</v>
+        <v>191</v>
       </c>
       <c r="G49" s="3" t="n">
         <v>0</v>
@@ -1897,10 +1910,10 @@
     </row>
     <row r="50" customHeight="1" ht="15" spans="1:10">
       <c r="A50" s="1" t="n">
-        <v>412075</v>
+        <v>412109</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>1</v>
@@ -1912,7 +1925,7 @@
         <v>3</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>910</v>
+        <v>819</v>
       </c>
       <c r="G50" s="3" t="n">
         <v>0</v>
@@ -1929,10 +1942,10 @@
     </row>
     <row r="51" customHeight="1" ht="15" spans="1:10">
       <c r="A51" s="1" t="n">
-        <v>412111</v>
+        <v>412092</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>1</v>
@@ -1944,7 +1957,7 @@
         <v>3</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>345</v>
+        <v>2553</v>
       </c>
       <c r="G51" s="3" t="n">
         <v>0</v>
@@ -1961,10 +1974,10 @@
     </row>
     <row r="52" customHeight="1" ht="15" spans="1:10">
       <c r="A52" s="1" t="n">
-        <v>412089</v>
+        <v>412366</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>1</v>
@@ -1976,7 +1989,7 @@
         <v>3</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>1100</v>
+        <v>1283</v>
       </c>
       <c r="G52" s="3" t="n">
         <v>0</v>
@@ -1993,10 +2006,10 @@
     </row>
     <row r="53" customHeight="1" ht="15" spans="1:10">
       <c r="A53" s="1" t="n">
-        <v>412126</v>
+        <v>412075</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>1</v>
@@ -2008,7 +2021,7 @@
         <v>3</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>21</v>
+        <v>910</v>
       </c>
       <c r="G53" s="3" t="n">
         <v>0</v>
@@ -2025,10 +2038,10 @@
     </row>
     <row r="54" customHeight="1" ht="15" spans="1:10">
       <c r="A54" s="1" t="n">
-        <v>701159</v>
+        <v>412111</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>1</v>
@@ -2040,7 +2053,7 @@
         <v>3</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>438</v>
+        <v>345</v>
       </c>
       <c r="G54" s="3" t="n">
         <v>0</v>
@@ -2057,10 +2070,10 @@
     </row>
     <row r="55" customHeight="1" ht="15" spans="1:10">
       <c r="A55" s="1" t="n">
-        <v>412139</v>
+        <v>412089</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>1</v>
@@ -2072,7 +2085,7 @@
         <v>3</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>520</v>
+        <v>1100</v>
       </c>
       <c r="G55" s="3" t="n">
         <v>0</v>
@@ -2089,10 +2102,10 @@
     </row>
     <row r="56" customHeight="1" ht="15" spans="1:10">
       <c r="A56" s="1" t="n">
-        <v>412108</v>
+        <v>412126</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>1</v>
@@ -2104,7 +2117,7 @@
         <v>3</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>600</v>
+        <v>21</v>
       </c>
       <c r="G56" s="3" t="n">
         <v>0</v>
@@ -2121,10 +2134,10 @@
     </row>
     <row r="57" customHeight="1" ht="15" spans="1:10">
       <c r="A57" s="1" t="n">
-        <v>412110</v>
+        <v>701159</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>1</v>
@@ -2136,7 +2149,7 @@
         <v>3</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>600</v>
+        <v>438</v>
       </c>
       <c r="G57" s="3" t="n">
         <v>0</v>
@@ -2153,10 +2166,10 @@
     </row>
     <row r="58" customHeight="1" ht="15" spans="1:10">
       <c r="A58" s="1" t="n">
-        <v>412033</v>
+        <v>412139</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>1</v>
@@ -2168,7 +2181,7 @@
         <v>3</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>600</v>
+        <v>520</v>
       </c>
       <c r="G58" s="3" t="n">
         <v>0</v>
@@ -2185,10 +2198,10 @@
     </row>
     <row r="59" customHeight="1" ht="15" spans="1:10">
       <c r="A59" s="1" t="n">
-        <v>412037</v>
+        <v>412108</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>1</v>
@@ -2217,33 +2230,129 @@
     </row>
     <row r="60" customHeight="1" ht="15" spans="1:10">
       <c r="A60" s="1" t="n">
+        <v>412110</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F60" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="G60" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" customHeight="1" ht="15" spans="1:10">
+      <c r="A61" s="1" t="n">
+        <v>412033</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="G61" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" customHeight="1" ht="15" spans="1:10">
+      <c r="A62" s="1" t="n">
+        <v>412037</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="G62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" customHeight="1" ht="15" spans="1:10">
+      <c r="A63" s="1" t="n">
         <v>813467</v>
       </c>
-      <c r="B60" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F60" s="3" t="n">
+      <c r="B63" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F63" s="3" t="n">
         <v>1271</v>
       </c>
-      <c r="G60" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H60" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I60" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J60" s="3" t="n">
+      <c r="G63" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" s="3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>